<commit_message>
feat(devis): feuille « Reçu de paiement » (quittance 50 % ou 100 %)
Nouvelle feuille reçu/facturation finale, dans le style de la maison :
- reprend automatiquement les infos du devis (n°, client, total TTC) ;
- nature du paiement (liste déroulante) : acompte 50 %, solde 50 %, paiement
  intégral 100 % ou montant libre ; mode de paiement (MVola, Orange/Airtel
  Money, virement, espèces) ;
- calcule le montant reçu, le reste à payer et le statut (✅ soldé / ⏳ reste) ;
- montant reçu écrit en toutes lettres (Ariary), automatique, via un 2e
  convertisseur ajouté à la feuille masquée « Lettres ».

Logo et recalcul à l'ouverture inclus. Script reproductible
scripts/devis-recu-paiement.py (étape 3 du pipeline).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012t79QaGVsNWbaZZyqFEvST
</commit_message>
<xml_diff>
--- a/docs/devis/OneWay_Devis_Transport.xlsx
+++ b/docs/devis/OneWay_Devis_Transport.xlsx
@@ -10,11 +10,13 @@
     <sheet name="⚙️ Paramètres" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="🧮 Calculateur Rapide" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="📊 Historique Devis" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lettres" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="🧾 Reçu de paiement" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Lettres" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="Vehicules">'⚙️ Paramètres'!$B$23:$B$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'📋 Devis Client'!$A$2:$J$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'🧾 Reçu de paiement'!$A$1:$J$37</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,12 +24,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0&quot; Ar&quot;"/>
     <numFmt numFmtId="165" formatCode="0&quot; L/100&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;+ &quot;0%"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="44">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -202,8 +205,90 @@
       <color rgb="001E3A5F"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00E07B20"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005B6B7F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F2937"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005B6B7F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="005B6B7F"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="005B6B7F"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -255,8 +340,28 @@
         <fgColor rgb="00F4F7FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002A4A72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E07B20"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF0F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -366,11 +471,60 @@
         <color rgb="00D9E1EC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E1EC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E1EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E1EC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E1EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E1EC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E1EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E1EC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E1EC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00D9E1EC"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -718,6 +872,74 @@
     <xf numFmtId="0" fontId="29" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="36" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -827,6 +1049,36 @@
         <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1238250" cy="1238250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1124,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="B1:I73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="0.5703125" customWidth="1" style="74" min="1" max="1"/>
@@ -2135,6 +2387,13 @@
         <f>"Arrêté le présent devis à la somme de "&amp;'Lettres'!$F$13&amp;" Ariary."</f>
         <v/>
       </c>
+      <c r="C53" s="121" t="n"/>
+      <c r="D53" s="121" t="n"/>
+      <c r="E53" s="121" t="n"/>
+      <c r="F53" s="121" t="n"/>
+      <c r="G53" s="121" t="n"/>
+      <c r="H53" s="121" t="n"/>
+      <c r="I53" s="122" t="n"/>
     </row>
     <row r="54" s="74">
       <c r="B54" s="92" t="n"/>
@@ -4592,10 +4851,426 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00128A4B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B3:I37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" style="74" min="1" max="1"/>
+    <col width="26" customWidth="1" style="74" min="2" max="2"/>
+    <col width="16" customWidth="1" style="74" min="3" max="3"/>
+    <col width="12" customWidth="1" style="74" min="4" max="4"/>
+    <col width="12" customWidth="1" style="74" min="5" max="5"/>
+    <col width="18" customWidth="1" style="74" min="6" max="6"/>
+    <col width="18" customWidth="1" style="74" min="7" max="7"/>
+    <col width="14" customWidth="1" style="74" min="8" max="8"/>
+    <col width="14" customWidth="1" style="74" min="9" max="9"/>
+    <col width="3" customWidth="1" style="74" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="18" customHeight="1" s="74"/>
+    <row r="3" ht="18" customHeight="1" s="74">
+      <c r="E3" s="123" t="inlineStr">
+        <is>
+          <t>REÇU DE PAIEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="74"/>
+    <row r="5" ht="18" customHeight="1" s="74">
+      <c r="E5" s="124" t="inlineStr">
+        <is>
+          <t>Transport · Livraison · Suivi Digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="74"/>
+    <row r="7" ht="6" customHeight="1" s="74"/>
+    <row r="8" ht="20" customHeight="1" s="74">
+      <c r="B8" s="125" t="inlineStr">
+        <is>
+          <t>N° REÇU :</t>
+        </is>
+      </c>
+      <c r="C8" s="126">
+        <f>"REC-"&amp;TEXT('⚙️ Paramètres'!C9,"0000")&amp;"-"&amp;TEXT(TODAY(),"MMYYYY")</f>
+        <v/>
+      </c>
+      <c r="E8" s="125" t="inlineStr">
+        <is>
+          <t>DATE :</t>
+        </is>
+      </c>
+      <c r="F8" s="127">
+        <f>TODAY()</f>
+        <v/>
+      </c>
+      <c r="G8" s="125" t="inlineStr">
+        <is>
+          <t>RÉF. DEVIS :</t>
+        </is>
+      </c>
+      <c r="H8" s="128">
+        <f>'📋 Devis Client'!C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="6" customHeight="1" s="74"/>
+    <row r="10" ht="20" customHeight="1" s="74">
+      <c r="B10" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  👤  CLIENT</t>
+        </is>
+      </c>
+      <c r="F10" s="130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🚛  ONE WAY — TRANSPORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="74">
+      <c r="B11" s="125" t="inlineStr">
+        <is>
+          <t>Nom / Société :</t>
+        </is>
+      </c>
+      <c r="C11" s="131">
+        <f>'📋 Devis Client'!C15</f>
+        <v/>
+      </c>
+      <c r="F11" s="125" t="inlineStr">
+        <is>
+          <t>Société :</t>
+        </is>
+      </c>
+      <c r="G11" s="131">
+        <f>'📋 Devis Client'!G15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="74">
+      <c r="B12" s="125" t="inlineStr">
+        <is>
+          <t>Adresse :</t>
+        </is>
+      </c>
+      <c r="C12" s="131">
+        <f>'📋 Devis Client'!C16</f>
+        <v/>
+      </c>
+      <c r="F12" s="125" t="inlineStr">
+        <is>
+          <t>Adresse :</t>
+        </is>
+      </c>
+      <c r="G12" s="131">
+        <f>'📋 Devis Client'!G16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="74">
+      <c r="B13" s="125" t="inlineStr">
+        <is>
+          <t>Ville :</t>
+        </is>
+      </c>
+      <c r="C13" s="131">
+        <f>'📋 Devis Client'!C17</f>
+        <v/>
+      </c>
+      <c r="F13" s="125" t="inlineStr">
+        <is>
+          <t>Téléphone :</t>
+        </is>
+      </c>
+      <c r="G13" s="131">
+        <f>'📋 Devis Client'!G17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="74">
+      <c r="B14" s="125" t="inlineStr">
+        <is>
+          <t>Téléphone :</t>
+        </is>
+      </c>
+      <c r="C14" s="131">
+        <f>'📋 Devis Client'!C18</f>
+        <v/>
+      </c>
+      <c r="F14" s="125" t="inlineStr">
+        <is>
+          <t>Email :</t>
+        </is>
+      </c>
+      <c r="G14" s="131">
+        <f>'📋 Devis Client'!G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="74">
+      <c r="B15" s="125" t="inlineStr">
+        <is>
+          <t>N° Client :</t>
+        </is>
+      </c>
+      <c r="C15" s="131">
+        <f>'📋 Devis Client'!C20</f>
+        <v/>
+      </c>
+      <c r="F15" s="125" t="inlineStr">
+        <is>
+          <t>MVola :</t>
+        </is>
+      </c>
+      <c r="G15" s="131">
+        <f>'📋 Devis Client'!G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="6" customHeight="1" s="74"/>
+    <row r="17" ht="22" customHeight="1" s="74">
+      <c r="B17" s="132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  💰  RÉCAPITULATIF DU RÈGLEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="19" customHeight="1" s="74">
+      <c r="B18" s="133" t="inlineStr">
+        <is>
+          <t>Montant total du devis (TTC)</t>
+        </is>
+      </c>
+      <c r="G18" s="134">
+        <f>'📋 Devis Client'!G52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="19" customHeight="1" s="74">
+      <c r="B19" s="135" t="inlineStr">
+        <is>
+          <t>Acompte — 50 % à la commande</t>
+        </is>
+      </c>
+      <c r="G19" s="134">
+        <f>ROUND('📋 Devis Client'!G52*0.5,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="19" customHeight="1" s="74">
+      <c r="B20" s="135" t="inlineStr">
+        <is>
+          <t>Solde — 50 % à la livraison</t>
+        </is>
+      </c>
+      <c r="G20" s="134">
+        <f>$G$18-$G$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="6" customHeight="1" s="74"/>
+    <row r="22" ht="22" customHeight="1" s="74">
+      <c r="B22" s="132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🧾  PAIEMENT REÇU</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="19" customHeight="1" s="74">
+      <c r="B23" s="136" t="inlineStr">
+        <is>
+          <t>Nature du paiement :</t>
+        </is>
+      </c>
+      <c r="G23" s="137" t="inlineStr">
+        <is>
+          <t>Acompte 50 % (à la commande)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="19" customHeight="1" s="74">
+      <c r="B24" s="136" t="inlineStr">
+        <is>
+          <t>Mode de paiement :</t>
+        </is>
+      </c>
+      <c r="G24" s="137" t="inlineStr">
+        <is>
+          <t>MVola</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1" s="74">
+      <c r="B25" s="136" t="inlineStr">
+        <is>
+          <t>Référence transaction :</t>
+        </is>
+      </c>
+      <c r="G25" s="137" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1" s="74">
+      <c r="B26" s="136" t="inlineStr">
+        <is>
+          <t>Montant libre (si nature = libre) :</t>
+        </is>
+      </c>
+      <c r="G26" s="138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="19" customHeight="1" s="74">
+      <c r="B27" s="136" t="inlineStr">
+        <is>
+          <t>Déjà encaissé (paiements précédents) :</t>
+        </is>
+      </c>
+      <c r="G27" s="138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1" s="74">
+      <c r="B28" s="139" t="inlineStr">
+        <is>
+          <t>💵  MONTANT REÇU (Ar) :</t>
+        </is>
+      </c>
+      <c r="G28" s="140">
+        <f>IF($G$23="Paiement intégral (100 %)",'📋 Devis Client'!G52,IF($G$23="Solde 50 % (à la livraison)",'📋 Devis Client'!G52-ROUND('📋 Devis Client'!G52*0.5,0),IF($G$23="Montant libre",$G$26,ROUND('📋 Devis Client'!G52*0.5,0))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1" s="74">
+      <c r="B29" s="120">
+        <f>"Reçu la somme de "&amp;'Lettres'!$I$13&amp;" Ariary."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="19" customHeight="1" s="74">
+      <c r="B30" s="133" t="inlineStr">
+        <is>
+          <t>Reste à payer après ce reçu :</t>
+        </is>
+      </c>
+      <c r="G30" s="134">
+        <f>ROUND(IF($G$23="Acompte 50 % (à la commande)",'📋 Devis Client'!G52-$G$28,IF($G$23="Montant libre",MAX('📋 Devis Client'!G52-$G$27-$G$28,0),0)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" s="74">
+      <c r="B31" s="128" t="inlineStr">
+        <is>
+          <t>Statut :</t>
+        </is>
+      </c>
+      <c r="G31" s="141">
+        <f>IF($G$30&lt;=0,"✅ SOLDÉ — Merci !","⏳ Reste à payer : "&amp;TEXT($G$30,"#,##0")&amp;" Ar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="8" customHeight="1" s="74"/>
+    <row r="33" ht="28" customHeight="1" s="74">
+      <c r="B33" s="142" t="inlineStr">
+        <is>
+          <t>Reçu valant quittance pour le montant ci-dessus, sous réserve d'encaissement. À conserver comme justificatif de paiement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="8" customHeight="1" s="74"/>
+    <row r="35" ht="46" customHeight="1" s="74">
+      <c r="B35" s="143" t="inlineStr">
+        <is>
+          <t>Le client</t>
+        </is>
+      </c>
+      <c r="F35" s="143" t="inlineStr">
+        <is>
+          <t>Pour One Way (cachet &amp; signature)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1" s="74">
+      <c r="B37" s="144" t="inlineStr">
+        <is>
+          <t>One Way SARL  ·  Transport · Livraison · Suivi Digital  ·  Antananarivo, Madagascar 🇲🇬</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="B22:I22"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="E3:I4"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="E5:I6"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B26:F26"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Acompte 50 % (à la commande),Solde 50 % (à la livraison),Paiement intégral (100 %),Montant libre"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"MVola,Orange Money,Airtel Money,Virement,Espèces"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1002"/>
+  <dimension ref="A1:I1002"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4613,6 +5288,15 @@
         <f>'📋 Devis Client'!$G$52</f>
         <v/>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="I1">
+        <f>'🧾 Reçu de paiement'!$G$28</f>
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4639,13 +5323,20 @@
         <f>INT(F1)</f>
         <v/>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="I2">
+        <f>INT(I1)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>0</v>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>g0</t>
@@ -4655,6 +5346,15 @@
         <f>MOD(F2,1000)</f>
         <v/>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>g0</t>
+        </is>
+      </c>
+      <c r="I3">
+        <f>MOD(I2,1000)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -4679,6 +5379,15 @@
         <f>MOD(INT(F2/1000),1000)</f>
         <v/>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="I4">
+        <f>MOD(INT(I2/1000),1000)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -4703,6 +5412,15 @@
         <f>MOD(INT(F2/1000000),1000)</f>
         <v/>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>g2</t>
+        </is>
+      </c>
+      <c r="I5">
+        <f>MOD(INT(I2/1000000),1000)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -4727,6 +5445,15 @@
         <f>MOD(INT(F2/1000000000),1000)</f>
         <v/>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>g3</t>
+        </is>
+      </c>
+      <c r="I6">
+        <f>MOD(INT(I2/1000000000),1000)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -4766,6 +5493,15 @@
         <f>IF(F3=0,"",INDEX($B$3:$B$1002,F3+1))</f>
         <v/>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>w0</t>
+        </is>
+      </c>
+      <c r="I8">
+        <f>IF(I3=0,"",INDEX($B$3:$B$1002,I3+1))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -4790,6 +5526,15 @@
         <f>IF(F4=0,"",IF(F4=1,"mille",INDEX($C$3:$C$1002,F4+1)&amp;" mille"))</f>
         <v/>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>w1</t>
+        </is>
+      </c>
+      <c r="I9">
+        <f>IF(I4=0,"",IF(I4=1,"mille",INDEX($C$3:$C$1002,I4+1)&amp;" mille"))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -4814,6 +5559,15 @@
         <f>IF(F5=0,"",INDEX($B$3:$B$1002,F5+1)&amp;IF(F5&gt;1," millions"," million"))</f>
         <v/>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>w2</t>
+        </is>
+      </c>
+      <c r="I10">
+        <f>IF(I5=0,"",INDEX($B$3:$B$1002,I5+1)&amp;IF(I5&gt;1," millions"," million"))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -4838,6 +5592,15 @@
         <f>IF(F6=0,"",INDEX($B$3:$B$1002,F6+1)&amp;IF(F6&gt;1," milliards"," milliard"))</f>
         <v/>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>w3</t>
+        </is>
+      </c>
+      <c r="I11">
+        <f>IF(I6=0,"",INDEX($B$3:$B$1002,I6+1)&amp;IF(I6&gt;1," milliards"," milliard"))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -4875,6 +5638,15 @@
       </c>
       <c r="F13">
         <f>IF(F2=0,"zéro",TRIM(F11&amp;" "&amp;F10&amp;" "&amp;F9&amp;" "&amp;F8))</f>
+        <v/>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>lettres</t>
+        </is>
+      </c>
+      <c r="I13">
+        <f>IF(I2=0,"zéro",TRIM(I11&amp;" "&amp;I10&amp;" "&amp;I9&amp;" "&amp;I8))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(devis): suivi des paiements (acompte/solde) dans la feuille Historique
Feuille « Historique Devis » étendue avec le suivi des règlements :
- colonnes ACOMPTE (Ar) et SOLDE (Ar) à saisir ;
- ENCAISSÉ, RESTE et PAIEMENT (✅ Soldé / ⏳ Partiel / ❌ Impayé, « — » si non
  accepté) calculés automatiquement ;
- ligne TOTAL et statistiques d'encaissement (total facturé / encaissé / reste,
  taux d'encaissement, nombre de devis soldés / partiels).

Zébrure, bordures et bandeaux (titre + stats) étendus jusqu'à la colonne Q.
Script reproductible scripts/historique-paiements.py (étape 4 du pipeline).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012t79QaGVsNWbaZZyqFEvST
</commit_message>
<xml_diff>
--- a/docs/devis/OneWay_Devis_Transport.xlsx
+++ b/docs/devis/OneWay_Devis_Transport.xlsx
@@ -16,6 +16,7 @@
   <definedNames>
     <definedName name="Vehicules">'⚙️ Paramètres'!$B$23:$B$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'📋 Devis Client'!$A$2:$J$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'📊 Historique Devis'!$A$1:$R$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'🧾 Reçu de paiement'!$A$1:$J$37</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -524,7 +525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -940,6 +941,7 @@
     <xf numFmtId="0" fontId="43" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1079,6 +1081,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -4304,7 +4309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L21"/>
+  <dimension ref="B2:Q26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="74" min="1" max="1"/>
@@ -4317,7 +4322,12 @@
     <col width="14" customWidth="1" style="74" min="9" max="10"/>
     <col width="13" customWidth="1" style="74" min="11" max="11"/>
     <col width="18" customWidth="1" style="74" min="12" max="12"/>
-    <col width="3" customWidth="1" style="74" min="13" max="13"/>
+    <col width="14" customWidth="1" style="74" min="13" max="13"/>
+    <col width="14" customWidth="1" style="74" min="14" max="14"/>
+    <col width="14" customWidth="1" style="74" min="15" max="15"/>
+    <col width="14" customWidth="1" style="74" min="16" max="16"/>
+    <col width="13" customWidth="1" style="74" min="17" max="17"/>
+    <col width="3" customWidth="1" style="74" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4386,6 +4396,31 @@
           <t>NOTES</t>
         </is>
       </c>
+      <c r="M6" s="103" t="inlineStr">
+        <is>
+          <t>ACOMPTE (Ar)</t>
+        </is>
+      </c>
+      <c r="N6" s="103" t="inlineStr">
+        <is>
+          <t>SOLDE (Ar)</t>
+        </is>
+      </c>
+      <c r="O6" s="103" t="inlineStr">
+        <is>
+          <t>ENCAISSÉ (Ar)</t>
+        </is>
+      </c>
+      <c r="P6" s="103" t="inlineStr">
+        <is>
+          <t>RESTE (Ar)</t>
+        </is>
+      </c>
+      <c r="Q6" s="103" t="inlineStr">
+        <is>
+          <t>PAIEMENT</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18.95" customHeight="1" s="74">
       <c r="B7" s="51" t="inlineStr">
@@ -4439,6 +4474,24 @@
           <t>Livraison OK</t>
         </is>
       </c>
+      <c r="M7" s="12" t="n">
+        <v>1441500</v>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>1441500</v>
+      </c>
+      <c r="O7" s="12">
+        <f>IF(K7&lt;&gt;"✅ Accepté","",N7+M7)</f>
+        <v/>
+      </c>
+      <c r="P7" s="12">
+        <f>IF(K7&lt;&gt;"✅ Accepté","",J7-M7-N7)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="62">
+        <f>IF(K7&lt;&gt;"✅ Accepté","—",IF(M7+N7&gt;=J7,"✅ Soldé",IF(M7+N7&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="18.95" customHeight="1" s="74">
       <c r="B8" s="53" t="inlineStr">
@@ -4492,6 +4545,24 @@
           <t>Marchandises générales</t>
         </is>
       </c>
+      <c r="M8" s="24" t="n">
+        <v>465500</v>
+      </c>
+      <c r="N8" s="24" t="n">
+        <v>465500</v>
+      </c>
+      <c r="O8" s="24">
+        <f>IF(K8&lt;&gt;"✅ Accepté","",N8+M8)</f>
+        <v/>
+      </c>
+      <c r="P8" s="24">
+        <f>IF(K8&lt;&gt;"✅ Accepté","",J8-M8-N8)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="65">
+        <f>IF(K8&lt;&gt;"✅ Accepté","—",IF(M8+N8&gt;=J8,"✅ Soldé",IF(M8+N8&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="18.95" customHeight="1" s="74">
       <c r="B9" s="51" t="inlineStr">
@@ -4545,6 +4616,22 @@
           <t>Périssables urgents</t>
         </is>
       </c>
+      <c r="M9" s="12" t="n">
+        <v>1889500</v>
+      </c>
+      <c r="N9" s="12" t="n"/>
+      <c r="O9" s="12">
+        <f>IF(K9&lt;&gt;"✅ Accepté","",N9+M9)</f>
+        <v/>
+      </c>
+      <c r="P9" s="12">
+        <f>IF(K9&lt;&gt;"✅ Accepté","",J9-M9-N9)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="62">
+        <f>IF(K9&lt;&gt;"✅ Accepté","—",IF(M9+N9&gt;=J9,"✅ Soldé",IF(M9+N9&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="18.95" customHeight="1" s="74">
       <c r="B10" s="53" t="inlineStr">
@@ -4598,6 +4685,22 @@
           <t>Semi-remorque</t>
         </is>
       </c>
+      <c r="M10" s="24" t="n">
+        <v>3289500</v>
+      </c>
+      <c r="N10" s="24" t="n"/>
+      <c r="O10" s="24">
+        <f>IF(K10&lt;&gt;"✅ Accepté","",N10+M10)</f>
+        <v/>
+      </c>
+      <c r="P10" s="24">
+        <f>IF(K10&lt;&gt;"✅ Accepté","",J10-M10-N10)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="65">
+        <f>IF(K10&lt;&gt;"✅ Accepté","—",IF(M10+N10&gt;=J10,"✅ Soldé",IF(M10+N10&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="18.95" customHeight="1" s="74">
       <c r="B11" s="51" t="inlineStr">
@@ -4651,6 +4754,20 @@
           <t>En cours</t>
         </is>
       </c>
+      <c r="M11" s="12" t="n"/>
+      <c r="N11" s="12" t="n"/>
+      <c r="O11" s="12">
+        <f>IF(K11&lt;&gt;"✅ Accepté","",N11+M11)</f>
+        <v/>
+      </c>
+      <c r="P11" s="12">
+        <f>IF(K11&lt;&gt;"✅ Accepté","",J11-M11-N11)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="62">
+        <f>IF(K11&lt;&gt;"✅ Accepté","—",IF(M11+N11&gt;=J11,"✅ Soldé",IF(M11+N11&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="18.95" customHeight="1" s="74">
       <c r="B12" s="53" t="inlineStr">
@@ -4704,6 +4821,20 @@
           <t>Prix refusé</t>
         </is>
       </c>
+      <c r="M12" s="24" t="n"/>
+      <c r="N12" s="24" t="n"/>
+      <c r="O12" s="24">
+        <f>IF(K12&lt;&gt;"✅ Accepté","",N12+M12)</f>
+        <v/>
+      </c>
+      <c r="P12" s="24">
+        <f>IF(K12&lt;&gt;"✅ Accepté","",J12-M12-N12)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="65">
+        <f>IF(K12&lt;&gt;"✅ Accepté","—",IF(M12+N12&gt;=J12,"✅ Soldé",IF(M12+N12&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="18.95" customHeight="1" s="74">
       <c r="B13" s="51" t="inlineStr">
@@ -4756,6 +4887,20 @@
         <is>
           <t>Devis émis</t>
         </is>
+      </c>
+      <c r="M13" s="12" t="n"/>
+      <c r="N13" s="12" t="n"/>
+      <c r="O13" s="12">
+        <f>IF(K13&lt;&gt;"✅ Accepté","",N13+M13)</f>
+        <v/>
+      </c>
+      <c r="P13" s="12">
+        <f>IF(K13&lt;&gt;"✅ Accepté","",J13-M13-N13)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="62">
+        <f>IF(K13&lt;&gt;"✅ Accepté","—",IF(M13+N13&gt;=J13,"✅ Soldé",IF(M13+N13&lt;=0,"❌ Impayé","⏳ Partiel")))</f>
+        <v/>
       </c>
     </row>
     <row r="14" ht="21.95" customHeight="1" s="74">
@@ -4774,6 +4919,23 @@
       </c>
       <c r="K14" s="28" t="n"/>
       <c r="L14" s="28" t="n"/>
+      <c r="M14" s="67">
+        <f>SUMIF($K$7:$K$13,"✅ Accepté",M7:M13)</f>
+        <v/>
+      </c>
+      <c r="N14" s="67">
+        <f>SUMIF($K$7:$K$13,"✅ Accepté",N7:N13)</f>
+        <v/>
+      </c>
+      <c r="O14" s="67">
+        <f>SUMIF($K$7:$K$13,"✅ Accepté",O7:O13)</f>
+        <v/>
+      </c>
+      <c r="P14" s="67">
+        <f>SUMIF($K$7:$K$13,"✅ Accepté",P7:P13)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="67" t="n"/>
     </row>
     <row r="16" ht="21.95" customHeight="1" s="74">
       <c r="B16" s="113" t="inlineStr">
@@ -4837,11 +4999,66 @@
         <v/>
       </c>
     </row>
+    <row r="22" ht="18.9" customHeight="1" s="74">
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>Total facturé (acceptés)</t>
+        </is>
+      </c>
+      <c r="C22" s="70">
+        <f>SUMIF($K$7:$K$13,"✅ Accepté",J7:J13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="18.9" customHeight="1" s="74">
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>Total encaissé</t>
+        </is>
+      </c>
+      <c r="C23" s="70">
+        <f>SUM(O7:O13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="18.9" customHeight="1" s="74">
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Reste à encaisser</t>
+        </is>
+      </c>
+      <c r="C24" s="70">
+        <f>SUMIF($K$7:$K$13,"✅ Accepté",P7:P13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="18.9" customHeight="1" s="74">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>Taux d'encaissement</t>
+        </is>
+      </c>
+      <c r="C25" s="69">
+        <f>IFERROR(C23/C22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="18.9" customHeight="1" s="74">
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>Devis soldés / partiels</t>
+        </is>
+      </c>
+      <c r="C26" s="108">
+        <f>COUNTIF(Q7:Q13,"✅ Soldé")&amp;" / "&amp;COUNTIF(Q7:Q13,"⏳ Partiel")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="B16:Q16"/>
     <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B2:L4"/>
+    <mergeCell ref="B2:Q4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
@@ -5090,6 +5307,8 @@
           <t>Acompte 50 % (à la commande)</t>
         </is>
       </c>
+      <c r="H23" s="121" t="n"/>
+      <c r="I23" s="122" t="n"/>
     </row>
     <row r="24" ht="19" customHeight="1" s="74">
       <c r="B24" s="136" t="inlineStr">
@@ -5102,6 +5321,8 @@
           <t>MVola</t>
         </is>
       </c>
+      <c r="H24" s="121" t="n"/>
+      <c r="I24" s="122" t="n"/>
     </row>
     <row r="25" ht="19" customHeight="1" s="74">
       <c r="B25" s="136" t="inlineStr">
@@ -5114,6 +5335,8 @@
           <t>—</t>
         </is>
       </c>
+      <c r="H25" s="121" t="n"/>
+      <c r="I25" s="122" t="n"/>
     </row>
     <row r="26" ht="19" customHeight="1" s="74">
       <c r="B26" s="136" t="inlineStr">
@@ -5124,6 +5347,8 @@
       <c r="G26" s="138" t="n">
         <v>0</v>
       </c>
+      <c r="H26" s="121" t="n"/>
+      <c r="I26" s="122" t="n"/>
     </row>
     <row r="27" ht="19" customHeight="1" s="74">
       <c r="B27" s="136" t="inlineStr">
@@ -5134,6 +5359,8 @@
       <c r="G27" s="138" t="n">
         <v>0</v>
       </c>
+      <c r="H27" s="121" t="n"/>
+      <c r="I27" s="122" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1" s="74">
       <c r="B28" s="139" t="inlineStr">
@@ -5151,6 +5378,13 @@
         <f>"Reçu la somme de "&amp;'Lettres'!$I$13&amp;" Ariary."</f>
         <v/>
       </c>
+      <c r="C29" s="121" t="n"/>
+      <c r="D29" s="121" t="n"/>
+      <c r="E29" s="121" t="n"/>
+      <c r="F29" s="121" t="n"/>
+      <c r="G29" s="121" t="n"/>
+      <c r="H29" s="121" t="n"/>
+      <c r="I29" s="122" t="n"/>
     </row>
     <row r="30" ht="19" customHeight="1" s="74">
       <c r="B30" s="133" t="inlineStr">
@@ -5189,11 +5423,17 @@
           <t>Le client</t>
         </is>
       </c>
+      <c r="C35" s="145" t="n"/>
+      <c r="D35" s="145" t="n"/>
+      <c r="E35" s="145" t="n"/>
       <c r="F35" s="143" t="inlineStr">
         <is>
           <t>Pour One Way (cachet &amp; signature)</t>
         </is>
       </c>
+      <c r="G35" s="145" t="n"/>
+      <c r="H35" s="145" t="n"/>
+      <c r="I35" s="145" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1" s="74">
       <c r="B37" s="144" t="inlineStr">
@@ -5214,8 +5454,8 @@
     <mergeCell ref="G30:I30"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B27:F27"/>
     <mergeCell ref="G15:I15"/>
-    <mergeCell ref="B27:F27"/>
     <mergeCell ref="G24:I24"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="G14:I14"/>

</xml_diff>